<commit_message>
<DKA - 03.09.2025> Added 10 experiments with thinner lines and sized panel.
</commit_message>
<xml_diff>
--- a/Experiments/Experiment Results.xlsx
+++ b/Experiments/Experiment Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deniz\AndroidStudioProjects\RoUtism\Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21824CE9-6C05-4AB2-AA72-5CBBF011444D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7756B2-CD19-46FF-90BF-50755FAD6FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{B0BE2EBB-2AC8-4FBA-BBB1-23CAB9B6C1A1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="52">
   <si>
     <t>Experiment No</t>
   </si>
@@ -132,6 +132,66 @@
   </si>
   <si>
     <t>Inference_1741637630398</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=x3ov9USxVxY</t>
+  </si>
+  <si>
+    <t>Inference_1741653121473</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=WuhpK7XgtG0</t>
+  </si>
+  <si>
+    <t>Inference_1741653707404</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ypDKx3vqnUU</t>
+  </si>
+  <si>
+    <t>Inference_1741653999003</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=OqKbl1mvJCo</t>
+  </si>
+  <si>
+    <t>Inference_1741655000143</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=wmAOe_klMKY</t>
+  </si>
+  <si>
+    <t>Inference_1741655942880</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=rc7VUoytoU4</t>
+  </si>
+  <si>
+    <t>Inference_1741656824816</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=UX_8Cy587jw</t>
+  </si>
+  <si>
+    <t>Inference_1741657082323</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=GQEhuVS7Wj8&amp;list=LL&amp;index=132</t>
+  </si>
+  <si>
+    <t>Inference_1741657547104</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=s1zL5AQqdl4</t>
+  </si>
+  <si>
+    <t>Inference_1741658247945</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=DZGN9fZvQhc</t>
+  </si>
+  <si>
+    <t>Inference_1741658767707</t>
   </si>
 </sst>
 </file>
@@ -648,11 +708,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDE0904B-8EC4-43AB-93D9-EEEB0BDBA96F}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="24.28515625" customWidth="1"/>
-    <col min="3" max="3" width="51.5703125" customWidth="1"/>
+    <col min="3" max="3" width="63.5703125" customWidth="1"/>
     <col min="4" max="4" width="17.42578125" customWidth="1"/>
     <col min="5" max="5" width="27.42578125" customWidth="1"/>
     <col min="6" max="6" width="39.28515625" customWidth="1"/>
@@ -912,6 +972,236 @@
         <v>3.08</v>
       </c>
     </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12">
+        <v>5.07</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14">
+        <v>5</v>
+      </c>
+      <c r="F14" t="s">
+        <v>37</v>
+      </c>
+      <c r="G14">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15">
+        <v>5</v>
+      </c>
+      <c r="F15" t="s">
+        <v>39</v>
+      </c>
+      <c r="G15">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17">
+        <v>4</v>
+      </c>
+      <c r="F17" t="s">
+        <v>43</v>
+      </c>
+      <c r="G17">
+        <v>4.1500000000000004</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18">
+        <v>4</v>
+      </c>
+      <c r="F18" t="s">
+        <v>45</v>
+      </c>
+      <c r="G18">
+        <v>1.46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19">
+        <v>5</v>
+      </c>
+      <c r="F19" t="s">
+        <v>47</v>
+      </c>
+      <c r="G19">
+        <v>4.51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20">
+        <v>5</v>
+      </c>
+      <c r="F20" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20">
+        <v>6.08</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21">
+        <v>5</v>
+      </c>
+      <c r="F21" t="s">
+        <v>51</v>
+      </c>
+      <c r="G21">
+        <v>0.56999999999999995</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
<03.11.2025 - DKA> Added 10 more experiments with several batches.
</commit_message>
<xml_diff>
--- a/Experiments/Experiment Results.xlsx
+++ b/Experiments/Experiment Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deniz\AndroidStudioProjects\RoUtism\Experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D7756B2-CD19-46FF-90BF-50755FAD6FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E316A3EC-78BF-4743-B605-99C506269381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{B0BE2EBB-2AC8-4FBA-BBB1-23CAB9B6C1A1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="74">
   <si>
     <t>Experiment No</t>
   </si>
@@ -192,13 +192,79 @@
   </si>
   <si>
     <t>Inference_1741658767707</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=xvB97P24GWg</t>
+  </si>
+  <si>
+    <t>Happy_Batch_1.zip</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=F6ZA7HMRfaU</t>
+  </si>
+  <si>
+    <t>Happy_Batch_2.zip</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bt7OERit4c8</t>
+  </si>
+  <si>
+    <t>Happy_Batch_3.zip</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=GMgsFZ4rkEI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=p1wCCTcg4zQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/shorts/3G2VX1xcxkc</t>
+  </si>
+  <si>
+    <t>Anxious_Batch_1.zip</t>
+  </si>
+  <si>
+    <t>Angry_Batch_1.zip</t>
+  </si>
+  <si>
+    <t>Angry_Batch_2.zip</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bnwLIdisr_Y</t>
+  </si>
+  <si>
+    <t>Sad_Batch_1.zip</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yGioU-bTuBY</t>
+  </si>
+  <si>
+    <t>Sad_Batch_2.zip</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=U9MIk0PVF7c</t>
+  </si>
+  <si>
+    <t>Angry_Batch_3.zip</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=V6veXwhlhsg</t>
+  </si>
+  <si>
+    <t>Happy_Batch_4.zip</t>
+  </si>
+  <si>
+    <t>Number of Batches</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -249,8 +315,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -290,6 +362,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
@@ -347,7 +425,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="8">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -356,8 +434,9 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="3"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1"/>
@@ -367,8 +446,10 @@
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="7"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="8" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="8">
+  <cellStyles count="9">
+    <cellStyle name="40% - Accent5" xfId="8" builtinId="47"/>
     <cellStyle name="Accent4" xfId="6" builtinId="41"/>
     <cellStyle name="Accent5" xfId="7" builtinId="45"/>
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -708,7 +789,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDE0904B-8EC4-43AB-93D9-EEEB0BDBA96F}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="24.28515625" customWidth="1"/>
@@ -716,10 +797,11 @@
     <col min="4" max="4" width="17.42578125" customWidth="1"/>
     <col min="5" max="5" width="27.42578125" customWidth="1"/>
     <col min="6" max="6" width="39.28515625" customWidth="1"/>
-    <col min="7" max="7" width="36.42578125" customWidth="1"/>
+    <col min="7" max="7" width="21" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -738,11 +820,14 @@
       <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -761,11 +846,14 @@
       <c r="F2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H2" s="6">
         <v>0.29097222222222224</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -784,11 +872,14 @@
       <c r="F3" t="s">
         <v>9</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H3">
         <v>4.49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -807,11 +898,14 @@
       <c r="F4" t="s">
         <v>12</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4">
         <v>5.04</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -830,11 +924,14 @@
       <c r="F5" t="s">
         <v>16</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H5">
         <v>9.4600000000000009</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -853,11 +950,14 @@
       <c r="F6" t="s">
         <v>18</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6">
         <v>6.13</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -876,11 +976,14 @@
       <c r="F7" t="s">
         <v>23</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H7">
         <v>4.24</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -899,11 +1002,14 @@
       <c r="F8" t="s">
         <v>26</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="s">
+        <v>73</v>
+      </c>
+      <c r="H8">
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -922,11 +1028,14 @@
       <c r="F9" t="s">
         <v>27</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H9">
         <v>5.43</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -945,11 +1054,14 @@
       <c r="F10" t="s">
         <v>30</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="s">
+        <v>73</v>
+      </c>
+      <c r="H10">
         <v>5.14</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -968,11 +1080,14 @@
       <c r="F11" t="s">
         <v>31</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11">
         <v>3.08</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -991,11 +1106,14 @@
       <c r="F12" t="s">
         <v>33</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12">
         <v>5.07</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1014,11 +1132,14 @@
       <c r="F13" t="s">
         <v>35</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="s">
+        <v>73</v>
+      </c>
+      <c r="H13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1037,11 +1158,14 @@
       <c r="F14" t="s">
         <v>37</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14">
         <v>2.08</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1060,11 +1184,14 @@
       <c r="F15" t="s">
         <v>39</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="s">
+        <v>73</v>
+      </c>
+      <c r="H15">
         <v>1.25</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1083,11 +1210,14 @@
       <c r="F16" t="s">
         <v>41</v>
       </c>
-      <c r="G16">
+      <c r="G16" t="s">
+        <v>73</v>
+      </c>
+      <c r="H16">
         <v>13.1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1106,11 +1236,14 @@
       <c r="F17" t="s">
         <v>43</v>
       </c>
-      <c r="G17">
+      <c r="G17" t="s">
+        <v>73</v>
+      </c>
+      <c r="H17">
         <v>4.1500000000000004</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1129,11 +1262,14 @@
       <c r="F18" t="s">
         <v>45</v>
       </c>
-      <c r="G18">
+      <c r="G18" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18">
         <v>1.46</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1152,11 +1288,14 @@
       <c r="F19" t="s">
         <v>47</v>
       </c>
-      <c r="G19">
+      <c r="G19" t="s">
+        <v>73</v>
+      </c>
+      <c r="H19">
         <v>4.51</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1175,11 +1314,14 @@
       <c r="F20" t="s">
         <v>49</v>
       </c>
-      <c r="G20">
+      <c r="G20" t="s">
+        <v>73</v>
+      </c>
+      <c r="H20">
         <v>6.08</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1198,11 +1340,275 @@
       <c r="F21" t="s">
         <v>51</v>
       </c>
-      <c r="G21">
+      <c r="G21" t="s">
+        <v>73</v>
+      </c>
+      <c r="H21">
         <v>0.56999999999999995</v>
       </c>
     </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22">
+        <v>4</v>
+      </c>
+      <c r="F22" t="s">
+        <v>53</v>
+      </c>
+      <c r="G22">
+        <v>347</v>
+      </c>
+      <c r="H22">
+        <v>5.46</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" t="s">
+        <v>54</v>
+      </c>
+      <c r="D23" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23">
+        <v>5</v>
+      </c>
+      <c r="F23" t="s">
+        <v>55</v>
+      </c>
+      <c r="G23">
+        <v>210</v>
+      </c>
+      <c r="H23">
+        <v>3.47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E24">
+        <v>4</v>
+      </c>
+      <c r="F24" t="s">
+        <v>57</v>
+      </c>
+      <c r="G24">
+        <v>382</v>
+      </c>
+      <c r="H24">
+        <v>6.18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" t="s">
+        <v>58</v>
+      </c>
+      <c r="D25" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25">
+        <v>5</v>
+      </c>
+      <c r="F25" t="s">
+        <v>61</v>
+      </c>
+      <c r="G25">
+        <v>20</v>
+      </c>
+      <c r="H25">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26">
+        <v>4</v>
+      </c>
+      <c r="F26" t="s">
+        <v>62</v>
+      </c>
+      <c r="G26">
+        <v>190</v>
+      </c>
+      <c r="H26">
+        <v>3.11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27">
+        <v>5</v>
+      </c>
+      <c r="F27" t="s">
+        <v>63</v>
+      </c>
+      <c r="G27">
+        <v>34</v>
+      </c>
+      <c r="H27">
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28">
+        <v>3</v>
+      </c>
+      <c r="F28" t="s">
+        <v>65</v>
+      </c>
+      <c r="G28">
+        <v>374</v>
+      </c>
+      <c r="H28">
+        <v>6.54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" t="s">
+        <v>22</v>
+      </c>
+      <c r="E29">
+        <v>4</v>
+      </c>
+      <c r="F29" t="s">
+        <v>67</v>
+      </c>
+      <c r="G29">
+        <v>174</v>
+      </c>
+      <c r="H29">
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" t="s">
+        <v>68</v>
+      </c>
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30">
+        <v>3</v>
+      </c>
+      <c r="F30" t="s">
+        <v>69</v>
+      </c>
+      <c r="G30">
+        <v>165</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" t="s">
+        <v>6</v>
+      </c>
+      <c r="E31">
+        <v>5</v>
+      </c>
+      <c r="F31" t="s">
+        <v>71</v>
+      </c>
+      <c r="G31">
+        <v>347</v>
+      </c>
+      <c r="H31">
+        <v>5.33</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>